<commit_message>
Expansion additions: add Shubham Housing Finance and WHP Jewellers (23 rows)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ABqraVRjb7dW9RHz2X61A
</commit_message>
<xml_diff>
--- a/tam/Zocket_Expansion_Additions.xlsx
+++ b/tam/Zocket_Expansion_Additions.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expansion List" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Expansion List'!$A$1:$W$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Expansion List'!$A$1:$W$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W22"/>
+  <dimension ref="A1:W23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1839,12 +1839,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Branch International Financial Services Pvt Ltd</t>
+          <t>Shubham Housing Development Finance Company Ltd</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>Shubham Housing Finance</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1854,23 +1854,23 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>NBFC &amp; Consumer Lending</t>
+          <t>Housing Finance</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://branch.co.in</t>
+          <t>https://www.shubham.co</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Karnataka</t>
+          <t>Haryana</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1879,10 +1879,10 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>832</v>
+        <v>824.1</v>
       </c>
       <c r="L14" t="n">
-        <v>97882353</v>
+        <v>96952941</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -1891,36 +1891,36 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>https://tracxn.com/d/legal-entities/india/branch-international-financial-services-private-limited/__d-H872WiN20gk3Rth1kQjhTc7pu2iy49u4e-85thrao</t>
+          <t>https://inc42.com/company/shubham-housing-development-finance-company/financials/</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>MNC – India-led</t>
+          <t>Indian private</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Branch International (US)</t>
+          <t>Independent (PE-backed)</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Branch app</t>
+          <t>Shubham</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Instant personal-loan app, 5 Cr+ Indian users</t>
+          <t>Affordable home loans to self-employed and low-income families via branch network</t>
         </is>
       </c>
       <c r="T14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>New – not in Apollo export</t>
+          <t>Apollo export – re-qualified (was dropped from TAM)</t>
         </is>
       </c>
     </row>
@@ -1944,38 +1944,38 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Automotive Manufacturers Pvt Ltd</t>
+          <t>Branch International Financial Services Pvt Ltd</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AMPL (Automotive Manufacturers)</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Automotive</t>
+          <t>BFSI</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Auto Dealerships</t>
+          <t>NBFC &amp; Consumer Lending</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.amplindia.com</t>
+          <t>https://branch.co.in</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Nagpur</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Maharashtra</t>
+          <t>Karnataka</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1984,57 +1984,57 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>11000</v>
+        <v>832</v>
       </c>
       <c r="L15" t="n">
-        <v>1294117647</v>
+        <v>97882353</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>https://www.crisilratings.com/mnt/winshare/Ratings/RatingList/RatingDocs/AutomotiveManufacturersPrivateLimited_May%2008_%202024_RR_343463.html</t>
+          <t>https://tracxn.com/d/legal-entities/india/branch-international-financial-services-private-limited/__d-H872WiN20gk3Rth1kQjhTc7pu2iy49u4e-85thrao</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Indian private</t>
+          <t>MNC – India-led</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>AMPL Group (Nagpur)</t>
+          <t>Branch International (US)</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Tata Motors CV dealerships, Mahindra, Maruti Suzuki, Bharat Petroleum outlets</t>
+          <t>Branch app</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Large multi-OEM vehicle retail dealer group (PV ~50% of revenue)</t>
+          <t>Instant personal-loan app, 5 Cr+ Indian users</t>
         </is>
       </c>
       <c r="T15" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Paid Media AI + Creative AI (dealer localisation)</t>
+          <t>Creative AI (AI Designer) + Brand Brain</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
@@ -2049,12 +2049,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>V.S.T. Motors Pvt Ltd</t>
+          <t>Automotive Manufacturers Pvt Ltd</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>VST Motors</t>
+          <t>AMPL (Automotive Manufacturers)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2069,18 +2069,18 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.vstmotors.com</t>
+          <t>https://www.amplindia.com</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Chennai</t>
+          <t>Nagpur</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Tamil Nadu</t>
+          <t>Maharashtra</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -2089,10 +2089,10 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>1741.9</v>
+        <v>11000</v>
       </c>
       <c r="L16" t="n">
-        <v>204929412</v>
+        <v>1294117647</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>https://www.icra.in/Rating/GetRationalReportFilePdf?Id=135496</t>
+          <t>https://www.crisilratings.com/mnt/winshare/Ratings/RatingList/RatingDocs/AutomotiveManufacturersPrivateLimited_May%2008_%202024_RR_343463.html</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -2116,21 +2116,21 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>VST Group (Chennai)</t>
+          <t>AMPL Group (Nagpur)</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Tata Motors CV, Kia, Jaguar Land Rover (VST &amp; Sons), Mercedes-Benz (VST Titanium Motors)</t>
+          <t>Tata Motors CV dealerships, Mahindra, Maruti Suzuki, Bharat Petroleum outlets</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Multi-OEM car &amp; CV retail dealer group selling to consumers</t>
+          <t>Large multi-OEM vehicle retail dealer group (PV ~50% of revenue)</t>
         </is>
       </c>
       <c r="T16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
@@ -2154,12 +2154,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Neon Motors Pvt Ltd</t>
+          <t>V.S.T. Motors Pvt Ltd</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Neon Motors</t>
+          <t>VST Motors</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2172,16 +2172,20 @@
           <t>Auto Dealerships</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://www.vstmotors.com</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
+          <t>Chennai</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Telangana</t>
+          <t>Tamil Nadu</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -2190,24 +2194,24 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>1247.6</v>
+        <v>1741.9</v>
       </c>
       <c r="L17" t="n">
-        <v>146776471</v>
+        <v>204929412</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>https://www.icra.in/Rating/GetRationalReportFilePdf?id=136174</t>
+          <t>https://www.icra.in/Rating/GetRationalReportFilePdf?Id=135496</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -2217,21 +2221,21 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Neon group (Independent)</t>
+          <t>VST Group (Chennai)</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Mahindra (PV &amp; CV), Hyundai, MG (Apple Cars)</t>
+          <t>Tata Motors CV, Kia, Jaguar Land Rover (VST &amp; Sons), Mercedes-Benz (VST Titanium Motors)</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Multi-brand car/CV retail dealer selling to consumers</t>
+          <t>Multi-OEM car &amp; CV retail dealer group selling to consumers</t>
         </is>
       </c>
       <c r="T17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
@@ -2255,12 +2259,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Star Automobiles</t>
+          <t>Neon Motors Pvt Ltd</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Star Automobiles (Mahindra / Hero)</t>
+          <t>Neon Motors</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2277,12 +2281,12 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Jabalpur</t>
+          <t>Hyderabad</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Madhya Pradesh</t>
+          <t>Telangana</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2291,10 +2295,10 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>990.6</v>
+        <v>1247.6</v>
       </c>
       <c r="L18" t="n">
-        <v>116541176</v>
+        <v>146776471</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -2303,7 +2307,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>https://www.icra.in/Rating/ShowRationalReportFilePdf/138597</t>
+          <t>https://www.icra.in/Rating/GetRationalReportFilePdf?id=136174</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -2318,25 +2322,25 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Star Group (Jabalpur)</t>
+          <t>Neon group (Independent)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Mahindra &amp; Mahindra PV/CV, Hero MotoCorp two-wheelers</t>
+          <t>Mahindra (PV &amp; CV), Hyundai, MG (Apple Cars)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Retail dealer of Mahindra vehicles and Hero two-wheelers to consumers</t>
+          <t>Multi-brand car/CV retail dealer selling to consumers</t>
         </is>
       </c>
       <c r="T18" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
@@ -2356,12 +2360,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Sree Krishna Automotives Hyd. Pvt Ltd</t>
+          <t>Star Automobiles</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Sree Krishna Automotives</t>
+          <t>Star Automobiles (Mahindra / Hero)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2378,12 +2382,12 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
+          <t>Jabalpur</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Telangana</t>
+          <t>Madhya Pradesh</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2392,10 +2396,10 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>912.7</v>
+        <v>990.6</v>
       </c>
       <c r="L19" t="n">
-        <v>107376471</v>
+        <v>116541176</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -2404,7 +2408,7 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>https://www.icra.in/Rating/GetRationalReportFilePdf?id=135354</t>
+          <t>https://www.icra.in/Rating/ShowRationalReportFilePdf/138597</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -2419,17 +2423,17 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Independent</t>
+          <t>Star Group (Jabalpur)</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Honda Cars, Jeep, Citroen, Ather, Jaguar Land Rover</t>
+          <t>Mahindra &amp; Mahindra PV/CV, Hero MotoCorp two-wheelers</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>Multi-brand car &amp; EV two-wheeler retail dealer</t>
+          <t>Retail dealer of Mahindra vehicles and Hero two-wheelers to consumers</t>
         </is>
       </c>
       <c r="T19" t="n">
@@ -2457,12 +2461,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>RNS Motors Pvt Ltd</t>
+          <t>Sree Krishna Automotives Hyd. Pvt Ltd</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>RNS Motors (Maruti Suzuki)</t>
+          <t>Sree Krishna Automotives</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2475,24 +2479,16 @@
           <t>Auto Dealerships</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>https://www.rnsmotors.com</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/rns-motors-pvt-ltd/</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Hyderabad</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Karnataka</t>
+          <t>Telangana</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2501,10 +2497,10 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>878.5</v>
+        <v>912.7</v>
       </c>
       <c r="L20" t="n">
-        <v>103352941</v>
+        <v>107376471</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2513,7 +2509,7 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>https://www.icra.in/Rating/GetRationalReportFilePdf?id=141778</t>
+          <t>https://www.icra.in/Rating/GetRationalReportFilePdf?id=135354</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -2528,17 +2524,17 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>RNS Group (R.N. Shetty family)</t>
+          <t>Independent</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>RNS Motors Arena, Nexa, True Value</t>
+          <t>Honda Cars, Jeep, Citroen, Ather, Jaguar Land Rover</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Authorised Maruti Suzuki retail dealer selling cars to consumers</t>
+          <t>Multi-brand car &amp; EV two-wheeler retail dealer</t>
         </is>
       </c>
       <c r="T20" t="n">
@@ -2566,12 +2562,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Lovely Autos</t>
+          <t>RNS Motors Pvt Ltd</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Lovely Autos (Maruti Suzuki / Bajaj)</t>
+          <t>RNS Motors (Maruti Suzuki)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2586,18 +2582,22 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.lovelyautos.com</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
+          <t>https://www.rnsmotors.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/rns-motors-pvt-ltd/</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Jalandhar</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Punjab</t>
+          <t>Karnataka</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2606,24 +2606,24 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>782.8</v>
+        <v>878.5</v>
       </c>
       <c r="L21" t="n">
-        <v>92088235</v>
+        <v>103352941</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>FY23</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>https://www.crisilratings.com/mnt/winshare/Ratings/RatingList/RatingDocs/LovelyAutos_September%2029,%202023_RR_326601.html</t>
+          <t>https://www.icra.in/Rating/GetRationalReportFilePdf?id=141778</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2633,21 +2633,21 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Lovely Group (Mittal family, Jalandhar)</t>
+          <t>RNS Group (R.N. Shetty family)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Maruti Suzuki, Bajaj Auto</t>
+          <t>RNS Motors Arena, Nexa, True Value</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Retail dealer of Maruti cars and Bajaj two-wheelers</t>
+          <t>Authorised Maruti Suzuki retail dealer selling cars to consumers</t>
         </is>
       </c>
       <c r="T21" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
@@ -2671,12 +2671,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Gargya Autocity Pvt Ltd</t>
+          <t>Lovely Autos</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Gargya Toyota</t>
+          <t>Lovely Autos (Maruti Suzuki / Bajaj)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2689,85 +2689,190 @@
           <t>Auto Dealerships</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>https://www.lovelyautos.com</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
+          <t>Jalandhar</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Punjab</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>782.8</v>
+      </c>
+      <c r="L22" t="n">
+        <v>92088235</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>FY23</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.crisilratings.com/mnt/winshare/Ratings/RatingList/RatingDocs/LovelyAutos_September%2029,%202023_RR_326601.html</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Indian private</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Lovely Group (Mittal family, Jalandhar)</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki, Bajaj Auto</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Retail dealer of Maruti cars and Bajaj two-wheelers</t>
+        </is>
+      </c>
+      <c r="T22" t="n">
+        <v>3</v>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>Paid Media AI + Creative AI (dealer localisation)</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>New – not in Apollo export</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Gargya Autocity Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Gargya Toyota</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Auto Dealerships</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>Guwahati</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>Assam</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="K22" t="n">
+      <c r="K23" t="n">
         <v>511.7</v>
       </c>
-      <c r="L22" t="n">
+      <c r="L23" t="n">
         <v>60200000</v>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="N22" s="2" t="inlineStr">
+      <c r="N23" s="2" t="inlineStr">
         <is>
           <t>https://www.icra.in/Rating/GetRationalReportFilePdf?Id=138870</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>Indian private</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>Gargya Group</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
+      <c r="R23" t="inlineStr">
         <is>
           <t>Toyota</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr">
+      <c r="S23" t="inlineStr">
         <is>
           <t>Toyota passenger-car retail dealer</t>
         </is>
       </c>
-      <c r="T22" t="n">
+      <c r="T23" t="n">
         <v>5</v>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="U23" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr">
+      <c r="V23" t="inlineStr">
         <is>
           <t>Paid Media AI + Creative AI (dealer localisation)</t>
         </is>
       </c>
-      <c r="W22" t="inlineStr">
+      <c r="W23" t="inlineStr">
         <is>
           <t>New – not in Apollo export</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W22"/>
+  <autoFilter ref="A1:W23"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
@@ -2799,14 +2904,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>